<commit_message>
docs: regenerate test catalog sau fix 6 gap HDSD
</commit_message>
<xml_diff>
--- a/docs/test_theo_hdsd_cu.xlsx
+++ b/docs/test_theo_hdsd_cu.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="930" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="930" uniqueCount="550">
   <si>
     <t>Mã TC</t>
   </si>
@@ -238,10 +238,7 @@
     <t>VB được ký số, hiển thị chữ ký trên PDF</t>
   </si>
   <si>
-    <t>⚠️ Partial</t>
-  </si>
-  <si>
-    <t>Backend endpoint có, UI end-to-end cần verify</t>
+    <t>Mock OTP flow — TODO tích hợp VNPT SmartCA SDK thực ở Phase 2</t>
   </si>
   <si>
     <t>TC-012</t>
@@ -844,616 +841,616 @@
     <t>VB gửi qua trục CP</t>
   </si>
   <si>
+    <t>Mock trục CP — TODO tích hợp thực Phase 2</t>
+  </si>
+  <si>
+    <t>TC-046</t>
+  </si>
+  <si>
+    <t>II.3.9</t>
+  </si>
+  <si>
+    <t>Chuyển lưu trữ VB đi</t>
+  </si>
+  <si>
+    <t>VB đã gửi</t>
+  </si>
+  <si>
+    <t>Chọn VB → Chuyển lưu trữ → Xác nhận</t>
+  </si>
+  <si>
+    <t>Form đầy đủ với Phòng/Kho lưu trữ</t>
+  </si>
+  <si>
+    <t>TC-047</t>
+  </si>
+  <si>
+    <t>II.3.10</t>
+  </si>
+  <si>
+    <t>Giao việc từ VB đi</t>
+  </si>
+  <si>
+    <t>VB đi đã duyệt</t>
+  </si>
+  <si>
+    <t>Chọn VB → Giao việc → chọn người</t>
+  </si>
+  <si>
+    <t>Task giao việc xuất hiện</t>
+  </si>
+  <si>
+    <t>TC-048</t>
+  </si>
+  <si>
+    <t>II.3.11</t>
+  </si>
+  <si>
+    <t>Thêm VB đi vào HSCV</t>
+  </si>
+  <si>
+    <t>Có HSCV active</t>
+  </si>
+  <si>
+    <t>VB vào HSCV</t>
+  </si>
+  <si>
+    <t>TC-049</t>
+  </si>
+  <si>
+    <t>II.3.12</t>
+  </si>
+  <si>
+    <t>Đánh dấu cá nhân VB đi</t>
+  </si>
+  <si>
+    <t>Chọn VB → Đánh dấu cá nhân → nhập ghi chú</t>
+  </si>
+  <si>
+    <t>Ghi chú lưu thành công</t>
+  </si>
+  <si>
+    <t>TC-050</t>
+  </si>
+  <si>
+    <t>II.3.13</t>
+  </si>
+  <si>
+    <t>Hủy duyệt VB đi</t>
+  </si>
+  <si>
+    <t>Chọn VB → Hủy duyệt → confirm</t>
+  </si>
+  <si>
+    <t>Status về pending</t>
+  </si>
+  <si>
+    <t>TC-051</t>
+  </si>
+  <si>
+    <t>II.4.1</t>
+  </si>
+  <si>
+    <t>VB liên thông</t>
+  </si>
+  <si>
+    <t>Chuyển về VB đến</t>
+  </si>
+  <si>
+    <t>VB liên thông status=received</t>
+  </si>
+  <si>
+    <t>Chọn VB → Chuyển về VB đến</t>
+  </si>
+  <si>
+    <t>Tạo VB đến mới, VB liên thông đánh dấu đã chuyển</t>
+  </si>
+  <si>
+    <t>TC-052</t>
+  </si>
+  <si>
+    <t>II.4.2</t>
+  </si>
+  <si>
+    <t>Tiếp nhận VB liên thông</t>
+  </si>
+  <si>
+    <t>VB chưa tiếp nhận</t>
+  </si>
+  <si>
+    <t>Chọn VB → Tiếp nhận</t>
+  </si>
+  <si>
+    <t>Status đổi sang received</t>
+  </si>
+  <si>
+    <t>TC-053</t>
+  </si>
+  <si>
+    <t>II.4.3</t>
+  </si>
+  <si>
+    <t>Từ chối VB liên thông</t>
+  </si>
+  <si>
+    <t>Chọn VB → Từ chối → nhập lý do → Xác nhận</t>
+  </si>
+  <si>
+    <t>VB chuyển về cơ quan gửi kèm lý do</t>
+  </si>
+  <si>
+    <t>TC-054</t>
+  </si>
+  <si>
+    <t>II.4.4</t>
+  </si>
+  <si>
+    <t>Xem chi tiết VB liên thông</t>
+  </si>
+  <si>
+    <t>Click vào dòng VB</t>
+  </si>
+  <si>
+    <t>Hiển thị chi tiết + status đúng</t>
+  </si>
+  <si>
+    <t>TC-055</t>
+  </si>
+  <si>
+    <t>II.4.5</t>
+  </si>
+  <si>
+    <t>Đồng ý thu hồi</t>
+  </si>
+  <si>
+    <t>VB status=recall_requested</t>
+  </si>
+  <si>
+    <t>Vào detail → click "Đồng ý thu hồi" → confirm</t>
+  </si>
+  <si>
+    <t>Status → recalled, VB đến liên kết soft-delete</t>
+  </si>
+  <si>
+    <t>TC-056</t>
+  </si>
+  <si>
+    <t>Từ chối thu hồi</t>
+  </si>
+  <si>
+    <t>Detail → "Từ chối thu hồi" → nhập lý do → Xác nhận</t>
+  </si>
+  <si>
+    <t>Status restore về trước recall, lưu lý do từ chối</t>
+  </si>
+  <si>
+    <t>TC-057</t>
+  </si>
+  <si>
+    <t>III.1.1</t>
+  </si>
+  <si>
+    <t>HSCV</t>
+  </si>
+  <si>
+    <t>Xem danh sách toàn bộ HSCV</t>
+  </si>
+  <si>
+    <t>Mở /ho-so-cong-viec</t>
+  </si>
+  <si>
+    <t>Hiển thị danh sách với filter theo status/keyword/ngày</t>
+  </si>
+  <si>
+    <t>TC-058</t>
+  </si>
+  <si>
+    <t>III.1.2</t>
+  </si>
+  <si>
+    <t>Thêm mới HSCV</t>
+  </si>
+  <si>
+    <t>Click Thêm → điền form (tên, loại VB, hạn, người phụ trách) → Xác nhận</t>
+  </si>
+  <si>
+    <t>HSCV xuất hiện trong danh sách</t>
+  </si>
+  <si>
+    <t>TC-059</t>
+  </si>
+  <si>
+    <t>III.1.3</t>
+  </si>
+  <si>
+    <t>Mở lại HSCV đã hoàn thành</t>
+  </si>
+  <si>
+    <t>HSCV status=4</t>
+  </si>
+  <si>
+    <t>Vào detail → click Mở lại → confirm</t>
+  </si>
+  <si>
+    <t>Status → 1 (đang xử lý), progress giữ 100</t>
+  </si>
+  <si>
+    <t>TC-060</t>
+  </si>
+  <si>
+    <t>III.1.4</t>
+  </si>
+  <si>
+    <t>Đánh dấu cá nhân HSCV</t>
+  </si>
+  <si>
+    <t>Có HSCV</t>
+  </si>
+  <si>
+    <t>Nhập ghi chú cá nhân → Lưu</t>
+  </si>
+  <si>
+    <t>Field "note" trên form HSCV</t>
+  </si>
+  <si>
+    <t>TC-061</t>
+  </si>
+  <si>
+    <t>III.1.5</t>
+  </si>
+  <si>
+    <t>Thêm cán bộ vào HSCV</t>
+  </si>
+  <si>
+    <t>Có HSCV + user khả dụng</t>
+  </si>
+  <si>
+    <t>Vào tab Phân công → chọn phòng ban → chọn user → Lưu</t>
+  </si>
+  <si>
+    <t>Cán bộ được thêm vào danh sách HSCV</t>
+  </si>
+  <si>
+    <t>TC-062</t>
+  </si>
+  <si>
+    <t>III.2.1</t>
+  </si>
+  <si>
+    <t>Xem HSCV chưa xử lý – phụ trách</t>
+  </si>
+  <si>
+    <t>Có HSCV user đang phụ trách</t>
+  </si>
+  <si>
+    <t>Mở /ho-so-cong-viec → tab Chưa XL phụ trách</t>
+  </si>
+  <si>
+    <t>Danh sách HSCV user đang phụ trách hiện ra</t>
+  </si>
+  <si>
+    <t>TC-063</t>
+  </si>
+  <si>
+    <t>III.2.2</t>
+  </si>
+  <si>
+    <t>Thêm HSCV từ tab chưa xử lý</t>
+  </si>
+  <si>
+    <t>Click Thêm → điền form → Xác nhận</t>
+  </si>
+  <si>
+    <t>HSCV mới tạo, user là người phụ trách</t>
+  </si>
+  <si>
+    <t>TC-064</t>
+  </si>
+  <si>
+    <t>III.2.3</t>
+  </si>
+  <si>
+    <t>Trình ký HSCV</t>
+  </si>
+  <si>
+    <t>HSCV status=1</t>
+  </si>
+  <si>
+    <t>Detail → click Trình ký → chọn lãnh đạo → Xác nhận</t>
+  </si>
+  <si>
+    <t>HSCV chuyển sang status trình ký</t>
+  </si>
+  <si>
+    <t>TC-065</t>
+  </si>
+  <si>
+    <t>III.2.4</t>
+  </si>
+  <si>
+    <t>Lấy số HSCV</t>
+  </si>
+  <si>
+    <t>HSCV status=1/3, chưa có số</t>
+  </si>
+  <si>
+    <t>Detail → Lấy số → chọn sổ văn bản → Xác nhận</t>
+  </si>
+  <si>
+    <t>Số cấp thành công, hiển thị số mới</t>
+  </si>
+  <si>
+    <t>Vừa implement quick-260418-hlj (reset theo năm)</t>
+  </si>
+  <si>
+    <t>TC-066</t>
+  </si>
+  <si>
+    <t>III.2.5</t>
+  </si>
+  <si>
+    <t>Hủy HSCV</t>
+  </si>
+  <si>
+    <t>HSCV đang xử lý</t>
+  </si>
+  <si>
+    <t>Detail → Hủy HSCV → confirm</t>
+  </si>
+  <si>
+    <t>HSCV chuyển status -3 (hủy)</t>
+  </si>
+  <si>
+    <t>Action hủy HSCV riêng với lý do</t>
+  </si>
+  <si>
+    <t>TC-067</t>
+  </si>
+  <si>
+    <t>III.2.6</t>
+  </si>
+  <si>
+    <t>Lưu / Gửi / Chuyển tiếp ý kiến</t>
+  </si>
+  <si>
+    <t>Detail → tab Ý kiến → chọn 1 trong 3 action → nhập nội dung → Xác nhận</t>
+  </si>
+  <si>
+    <t>Ý kiến lưu + gửi thành công</t>
+  </si>
+  <si>
+    <t>Chuyển tiếp ý kiến cho user review</t>
+  </si>
+  <si>
+    <t>TC-068</t>
+  </si>
+  <si>
+    <t>III.2</t>
+  </si>
+  <si>
+    <t>Chuyển tiếp HSCV cho người khác</t>
+  </si>
+  <si>
+    <t>HSCV đang phụ trách</t>
+  </si>
+  <si>
+    <t>Chuyển tiếp HSCV sang user khác xử lý</t>
+  </si>
+  <si>
+    <t>Người mới trở thành phụ trách</t>
+  </si>
+  <si>
+    <t>Transfer ownership HSCV (same unit)</t>
+  </si>
+  <si>
+    <t>TC-069</t>
+  </si>
+  <si>
+    <t>III.3.1</t>
+  </si>
+  <si>
+    <t>Cấu hình ngoại giao / gửi nhanh</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Mở /cau-hinh-gui-nhanh → chọn user vào danh sách quick-recipient → Lưu</t>
+  </si>
+  <si>
+    <t>Danh sách user lưu, khi gửi VB tự tick sẵn</t>
+  </si>
+  <si>
+    <t>🚫 Hidden</t>
+  </si>
+  <si>
+    <t>Ẩn Phase 1 — flag off. Code còn, chờ Phase 2 bật</t>
+  </si>
+  <si>
+    <t>TC-070</t>
+  </si>
+  <si>
+    <t>III.4.1</t>
+  </si>
+  <si>
+    <t>Giao diện tổng quan công việc</t>
+  </si>
+  <si>
+    <t>Admin/Lãnh đạo</t>
+  </si>
+  <si>
+    <t>Mở Dashboard / Kiểm soát công việc</t>
+  </si>
+  <si>
+    <t>Dashboard tổng quan HSCV hiển thị KPI + chart</t>
+  </si>
+  <si>
+    <t>Gộp vào /dashboard chung — thống nhất với user</t>
+  </si>
+  <si>
+    <t>TC-071</t>
+  </si>
+  <si>
+    <t>III.4.2</t>
+  </si>
+  <si>
+    <t>Thống kê công việc theo đơn vị</t>
+  </si>
+  <si>
+    <t>Mở /ho-so-cong-viec/bao-cao</t>
+  </si>
+  <si>
+    <t>Báo cáo thống kê theo đơn vị/cán bộ + charts</t>
+  </si>
+  <si>
+    <t>TC-072</t>
+  </si>
+  <si>
+    <t>IV.1.1</t>
+  </si>
+  <si>
+    <t>Quản trị</t>
+  </si>
+  <si>
+    <t>Danh sách phòng ban - người dùng</t>
+  </si>
+  <si>
+    <t>Mở /quan-tri/nguoi-dung</t>
+  </si>
+  <si>
+    <t>Tree phòng ban bên trái + table người dùng bên phải</t>
+  </si>
+  <si>
+    <t>TC-073</t>
+  </si>
+  <si>
+    <t>IV.1.2</t>
+  </si>
+  <si>
+    <t>Thêm mới đơn vị/phòng ban</t>
+  </si>
+  <si>
+    <t>/quan-tri/don-vi → Thêm → điền name/code/parent → Lưu</t>
+  </si>
+  <si>
+    <t>Phòng ban xuất hiện trong tree</t>
+  </si>
+  <si>
+    <t>TC-074</t>
+  </si>
+  <si>
+    <t>IV.1.3</t>
+  </si>
+  <si>
+    <t>Thêm mới người dùng</t>
+  </si>
+  <si>
+    <t>Admin, có phòng ban</t>
+  </si>
+  <si>
+    <t>Chọn phòng ban → Thêm người dùng → điền form → Lưu</t>
+  </si>
+  <si>
+    <t>User tạo thành công, password mặc định Admin@123</t>
+  </si>
+  <si>
+    <t>TC-075</t>
+  </si>
+  <si>
+    <t>IV.1.4</t>
+  </si>
+  <si>
+    <t>Cập nhật thông tin phòng ban</t>
+  </si>
+  <si>
+    <t>Có phòng ban</t>
+  </si>
+  <si>
+    <t>Chọn phòng ban → Sửa → update thông tin → Lưu</t>
+  </si>
+  <si>
+    <t>Phòng ban update</t>
+  </si>
+  <si>
+    <t>TC-076</t>
+  </si>
+  <si>
+    <t>IV.1.5</t>
+  </si>
+  <si>
+    <t>Cập nhật thông tin người dùng</t>
+  </si>
+  <si>
+    <t>Có user</t>
+  </si>
+  <si>
+    <t>Chọn user → Sửa → update → Lưu</t>
+  </si>
+  <si>
+    <t>User info update</t>
+  </si>
+  <si>
+    <t>Không update username/password từ endpoint này</t>
+  </si>
+  <si>
+    <t>TC-077</t>
+  </si>
+  <si>
+    <t>IV.1.6</t>
+  </si>
+  <si>
+    <t>Xóa phòng ban</t>
+  </si>
+  <si>
+    <t>Phòng ban không có user/child</t>
+  </si>
+  <si>
+    <t>Chọn phòng ban → Xóa → confirm</t>
+  </si>
+  <si>
+    <t>Phòng ban xóa khỏi tree</t>
+  </si>
+  <si>
+    <t>Check constraint trước xóa</t>
+  </si>
+  <si>
+    <t>TC-078</t>
+  </si>
+  <si>
+    <t>IV.1.7</t>
+  </si>
+  <si>
+    <t>Xóa người dùng</t>
+  </si>
+  <si>
+    <t>User không đang phụ trách task</t>
+  </si>
+  <si>
+    <t>Chọn user → Xóa → confirm</t>
+  </si>
+  <si>
+    <t>User soft-delete</t>
+  </si>
+  <si>
+    <t>TC-079</t>
+  </si>
+  <si>
+    <t>IV.1.8</t>
+  </si>
+  <si>
+    <t>Giới hạn quyền cho đơn vị</t>
+  </si>
+  <si>
+    <t>Chọn đơn vị → Giới hạn quyền → chọn rights → Lưu</t>
+  </si>
+  <si>
+    <t>Quyền tối đa cho đơn vị set, user trong đơn vị không vượt quyền</t>
+  </si>
+  <si>
     <t>❌ Missing</t>
   </si>
   <si>
-    <t>HDSD có, code chưa có endpoint riêng — hỏi nghiệp vụ</t>
-  </si>
-  <si>
-    <t>TC-046</t>
-  </si>
-  <si>
-    <t>II.3.9</t>
-  </si>
-  <si>
-    <t>Chuyển lưu trữ VB đi</t>
-  </si>
-  <si>
-    <t>VB đã gửi</t>
-  </si>
-  <si>
-    <t>Chọn VB → Chuyển lưu trữ → Xác nhận</t>
-  </si>
-  <si>
-    <t>Có endpoint, thiếu form phòng/kho lưu trữ đầy đủ</t>
-  </si>
-  <si>
-    <t>TC-047</t>
-  </si>
-  <si>
-    <t>II.3.10</t>
-  </si>
-  <si>
-    <t>Giao việc từ VB đi</t>
-  </si>
-  <si>
-    <t>VB đi đã duyệt</t>
-  </si>
-  <si>
-    <t>Chọn VB → Giao việc → chọn người</t>
-  </si>
-  <si>
-    <t>Task giao việc xuất hiện</t>
-  </si>
-  <si>
-    <t>TC-048</t>
-  </si>
-  <si>
-    <t>II.3.11</t>
-  </si>
-  <si>
-    <t>Thêm VB đi vào HSCV</t>
-  </si>
-  <si>
-    <t>Có HSCV active</t>
-  </si>
-  <si>
-    <t>VB vào HSCV</t>
-  </si>
-  <si>
-    <t>TC-049</t>
-  </si>
-  <si>
-    <t>II.3.12</t>
-  </si>
-  <si>
-    <t>Đánh dấu cá nhân VB đi</t>
-  </si>
-  <si>
-    <t>Chọn VB → Đánh dấu cá nhân → nhập ghi chú</t>
-  </si>
-  <si>
-    <t>Ghi chú lưu thành công</t>
-  </si>
-  <si>
-    <t>TC-050</t>
-  </si>
-  <si>
-    <t>II.3.13</t>
-  </si>
-  <si>
-    <t>Hủy duyệt VB đi</t>
-  </si>
-  <si>
-    <t>Chọn VB → Hủy duyệt → confirm</t>
-  </si>
-  <si>
-    <t>Status về pending</t>
-  </si>
-  <si>
-    <t>TC-051</t>
-  </si>
-  <si>
-    <t>II.4.1</t>
-  </si>
-  <si>
-    <t>VB liên thông</t>
-  </si>
-  <si>
-    <t>Chuyển về VB đến</t>
-  </si>
-  <si>
-    <t>VB liên thông status=received</t>
-  </si>
-  <si>
-    <t>Chọn VB → Chuyển về VB đến</t>
-  </si>
-  <si>
-    <t>Tạo VB đến mới, VB liên thông đánh dấu đã chuyển</t>
-  </si>
-  <si>
-    <t>TC-052</t>
-  </si>
-  <si>
-    <t>II.4.2</t>
-  </si>
-  <si>
-    <t>Tiếp nhận VB liên thông</t>
-  </si>
-  <si>
-    <t>VB chưa tiếp nhận</t>
-  </si>
-  <si>
-    <t>Chọn VB → Tiếp nhận</t>
-  </si>
-  <si>
-    <t>Status đổi sang received</t>
-  </si>
-  <si>
-    <t>TC-053</t>
-  </si>
-  <si>
-    <t>II.4.3</t>
-  </si>
-  <si>
-    <t>Từ chối VB liên thông</t>
-  </si>
-  <si>
-    <t>Chọn VB → Từ chối → nhập lý do → Xác nhận</t>
-  </si>
-  <si>
-    <t>VB chuyển về cơ quan gửi kèm lý do</t>
-  </si>
-  <si>
-    <t>TC-054</t>
-  </si>
-  <si>
-    <t>II.4.4</t>
-  </si>
-  <si>
-    <t>Xem chi tiết VB liên thông</t>
-  </si>
-  <si>
-    <t>Click vào dòng VB</t>
-  </si>
-  <si>
-    <t>Hiển thị chi tiết + status đúng</t>
-  </si>
-  <si>
-    <t>TC-055</t>
-  </si>
-  <si>
-    <t>II.4.5</t>
-  </si>
-  <si>
-    <t>Đồng ý thu hồi</t>
-  </si>
-  <si>
-    <t>VB status=recall_requested</t>
-  </si>
-  <si>
-    <t>Vào detail → click "Đồng ý thu hồi" → confirm</t>
-  </si>
-  <si>
-    <t>Status → recalled, VB đến liên kết soft-delete</t>
-  </si>
-  <si>
-    <t>TC-056</t>
-  </si>
-  <si>
-    <t>Từ chối thu hồi</t>
-  </si>
-  <si>
-    <t>Detail → "Từ chối thu hồi" → nhập lý do → Xác nhận</t>
-  </si>
-  <si>
-    <t>Status restore về trước recall, lưu lý do từ chối</t>
-  </si>
-  <si>
-    <t>TC-057</t>
-  </si>
-  <si>
-    <t>III.1.1</t>
-  </si>
-  <si>
-    <t>HSCV</t>
-  </si>
-  <si>
-    <t>Xem danh sách toàn bộ HSCV</t>
-  </si>
-  <si>
-    <t>Mở /ho-so-cong-viec</t>
-  </si>
-  <si>
-    <t>Hiển thị danh sách với filter theo status/keyword/ngày</t>
-  </si>
-  <si>
-    <t>TC-058</t>
-  </si>
-  <si>
-    <t>III.1.2</t>
-  </si>
-  <si>
-    <t>Thêm mới HSCV</t>
-  </si>
-  <si>
-    <t>Click Thêm → điền form (tên, loại VB, hạn, người phụ trách) → Xác nhận</t>
-  </si>
-  <si>
-    <t>HSCV xuất hiện trong danh sách</t>
-  </si>
-  <si>
-    <t>TC-059</t>
-  </si>
-  <si>
-    <t>III.1.3</t>
-  </si>
-  <si>
-    <t>Mở lại HSCV đã hoàn thành</t>
-  </si>
-  <si>
-    <t>HSCV status=4</t>
-  </si>
-  <si>
-    <t>Vào detail → click Mở lại → confirm</t>
-  </si>
-  <si>
-    <t>Status → 1 (đang xử lý), progress giữ 100</t>
-  </si>
-  <si>
-    <t>TC-060</t>
-  </si>
-  <si>
-    <t>III.1.4</t>
-  </si>
-  <si>
-    <t>Đánh dấu cá nhân HSCV</t>
-  </si>
-  <si>
-    <t>Có HSCV</t>
-  </si>
-  <si>
-    <t>Nhập ghi chú cá nhân → Lưu</t>
-  </si>
-  <si>
-    <t>Field "note" trên form HSCV</t>
-  </si>
-  <si>
-    <t>TC-061</t>
-  </si>
-  <si>
-    <t>III.1.5</t>
-  </si>
-  <si>
-    <t>Thêm cán bộ vào HSCV</t>
-  </si>
-  <si>
-    <t>Có HSCV + user khả dụng</t>
-  </si>
-  <si>
-    <t>Vào tab Phân công → chọn phòng ban → chọn user → Lưu</t>
-  </si>
-  <si>
-    <t>Cán bộ được thêm vào danh sách HSCV</t>
-  </si>
-  <si>
-    <t>TC-062</t>
-  </si>
-  <si>
-    <t>III.2.1</t>
-  </si>
-  <si>
-    <t>Xem HSCV chưa xử lý – phụ trách</t>
-  </si>
-  <si>
-    <t>Có HSCV user đang phụ trách</t>
-  </si>
-  <si>
-    <t>Mở /ho-so-cong-viec → tab Chưa XL phụ trách</t>
-  </si>
-  <si>
-    <t>Danh sách HSCV user đang phụ trách hiện ra</t>
-  </si>
-  <si>
-    <t>TC-063</t>
-  </si>
-  <si>
-    <t>III.2.2</t>
-  </si>
-  <si>
-    <t>Thêm HSCV từ tab chưa xử lý</t>
-  </si>
-  <si>
-    <t>Click Thêm → điền form → Xác nhận</t>
-  </si>
-  <si>
-    <t>HSCV mới tạo, user là người phụ trách</t>
-  </si>
-  <si>
-    <t>TC-064</t>
-  </si>
-  <si>
-    <t>III.2.3</t>
-  </si>
-  <si>
-    <t>Trình ký HSCV</t>
-  </si>
-  <si>
-    <t>HSCV status=1</t>
-  </si>
-  <si>
-    <t>Detail → click Trình ký → chọn lãnh đạo → Xác nhận</t>
-  </si>
-  <si>
-    <t>HSCV chuyển sang status trình ký</t>
-  </si>
-  <si>
-    <t>TC-065</t>
-  </si>
-  <si>
-    <t>III.2.4</t>
-  </si>
-  <si>
-    <t>Lấy số HSCV</t>
-  </si>
-  <si>
-    <t>HSCV status=1/3, chưa có số</t>
-  </si>
-  <si>
-    <t>Detail → Lấy số → chọn sổ văn bản → Xác nhận</t>
-  </si>
-  <si>
-    <t>Số cấp thành công, hiển thị số mới</t>
-  </si>
-  <si>
-    <t>Vừa implement quick-260418-hlj (reset theo năm)</t>
-  </si>
-  <si>
-    <t>TC-066</t>
-  </si>
-  <si>
-    <t>III.2.5</t>
-  </si>
-  <si>
-    <t>Hủy HSCV</t>
-  </si>
-  <si>
-    <t>HSCV đang xử lý</t>
-  </si>
-  <si>
-    <t>Detail → Hủy HSCV → confirm</t>
-  </si>
-  <si>
-    <t>HSCV chuyển status -3 (hủy)</t>
-  </si>
-  <si>
-    <t>Dùng chung change-status thay vì action riêng</t>
-  </si>
-  <si>
-    <t>TC-067</t>
-  </si>
-  <si>
-    <t>III.2.6</t>
-  </si>
-  <si>
-    <t>Lưu / Gửi / Chuyển tiếp ý kiến</t>
-  </si>
-  <si>
-    <t>Detail → tab Ý kiến → chọn 1 trong 3 action → nhập nội dung → Xác nhận</t>
-  </si>
-  <si>
-    <t>Ý kiến lưu + gửi thành công</t>
-  </si>
-  <si>
-    <t>Có Lưu + Gửi. Thiếu "Chuyển tiếp" (forward to user khác)</t>
-  </si>
-  <si>
-    <t>TC-068</t>
-  </si>
-  <si>
-    <t>III.2</t>
-  </si>
-  <si>
-    <t>Chuyển tiếp HSCV cho người khác</t>
-  </si>
-  <si>
-    <t>HSCV đang phụ trách</t>
-  </si>
-  <si>
-    <t>Chuyển tiếp HSCV sang user khác xử lý</t>
-  </si>
-  <si>
-    <t>Người mới trở thành phụ trách</t>
-  </si>
-  <si>
-    <t>HDSD có, code chỉ có assign staff (phân công)</t>
-  </si>
-  <si>
-    <t>TC-069</t>
-  </si>
-  <si>
-    <t>III.3.1</t>
-  </si>
-  <si>
-    <t>Cấu hình ngoại giao / gửi nhanh</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>Mở /cau-hinh-gui-nhanh → chọn user vào danh sách quick-recipient → Lưu</t>
-  </si>
-  <si>
-    <t>Danh sách user lưu, khi gửi VB tự tick sẵn</t>
-  </si>
-  <si>
-    <t>🚫 Hidden</t>
-  </si>
-  <si>
-    <t>Ẩn Phase 1 — flag off. Code còn, chờ Phase 2 bật</t>
-  </si>
-  <si>
-    <t>TC-070</t>
-  </si>
-  <si>
-    <t>III.4.1</t>
-  </si>
-  <si>
-    <t>Giao diện tổng quan công việc</t>
-  </si>
-  <si>
-    <t>Admin/Lãnh đạo</t>
-  </si>
-  <si>
-    <t>Mở Dashboard / Kiểm soát công việc</t>
-  </si>
-  <si>
-    <t>Dashboard tổng quan HSCV hiển thị KPI + chart</t>
-  </si>
-  <si>
-    <t>Gộp vào /dashboard chung, không có trang riêng</t>
-  </si>
-  <si>
-    <t>TC-071</t>
-  </si>
-  <si>
-    <t>III.4.2</t>
-  </si>
-  <si>
-    <t>Thống kê công việc theo đơn vị</t>
-  </si>
-  <si>
-    <t>Mở /ho-so-cong-viec/bao-cao</t>
-  </si>
-  <si>
-    <t>Báo cáo thống kê theo đơn vị/cán bộ + charts</t>
-  </si>
-  <si>
-    <t>TC-072</t>
-  </si>
-  <si>
-    <t>IV.1.1</t>
-  </si>
-  <si>
-    <t>Quản trị</t>
-  </si>
-  <si>
-    <t>Danh sách phòng ban - người dùng</t>
-  </si>
-  <si>
-    <t>Mở /quan-tri/nguoi-dung</t>
-  </si>
-  <si>
-    <t>Tree phòng ban bên trái + table người dùng bên phải</t>
-  </si>
-  <si>
-    <t>TC-073</t>
-  </si>
-  <si>
-    <t>IV.1.2</t>
-  </si>
-  <si>
-    <t>Thêm mới đơn vị/phòng ban</t>
-  </si>
-  <si>
-    <t>/quan-tri/don-vi → Thêm → điền name/code/parent → Lưu</t>
-  </si>
-  <si>
-    <t>Phòng ban xuất hiện trong tree</t>
-  </si>
-  <si>
-    <t>TC-074</t>
-  </si>
-  <si>
-    <t>IV.1.3</t>
-  </si>
-  <si>
-    <t>Thêm mới người dùng</t>
-  </si>
-  <si>
-    <t>Admin, có phòng ban</t>
-  </si>
-  <si>
-    <t>Chọn phòng ban → Thêm người dùng → điền form → Lưu</t>
-  </si>
-  <si>
-    <t>User tạo thành công, password mặc định Admin@123</t>
-  </si>
-  <si>
-    <t>TC-075</t>
-  </si>
-  <si>
-    <t>IV.1.4</t>
-  </si>
-  <si>
-    <t>Cập nhật thông tin phòng ban</t>
-  </si>
-  <si>
-    <t>Có phòng ban</t>
-  </si>
-  <si>
-    <t>Chọn phòng ban → Sửa → update thông tin → Lưu</t>
-  </si>
-  <si>
-    <t>Phòng ban update</t>
-  </si>
-  <si>
-    <t>TC-076</t>
-  </si>
-  <si>
-    <t>IV.1.5</t>
-  </si>
-  <si>
-    <t>Cập nhật thông tin người dùng</t>
-  </si>
-  <si>
-    <t>Có user</t>
-  </si>
-  <si>
-    <t>Chọn user → Sửa → update → Lưu</t>
-  </si>
-  <si>
-    <t>User info update</t>
-  </si>
-  <si>
-    <t>Không update username/password từ endpoint này</t>
-  </si>
-  <si>
-    <t>TC-077</t>
-  </si>
-  <si>
-    <t>IV.1.6</t>
-  </si>
-  <si>
-    <t>Xóa phòng ban</t>
-  </si>
-  <si>
-    <t>Phòng ban không có user/child</t>
-  </si>
-  <si>
-    <t>Chọn phòng ban → Xóa → confirm</t>
-  </si>
-  <si>
-    <t>Phòng ban xóa khỏi tree</t>
-  </si>
-  <si>
-    <t>Check constraint trước xóa</t>
-  </si>
-  <si>
-    <t>TC-078</t>
-  </si>
-  <si>
-    <t>IV.1.7</t>
-  </si>
-  <si>
-    <t>Xóa người dùng</t>
-  </si>
-  <si>
-    <t>User không đang phụ trách task</t>
-  </si>
-  <si>
-    <t>Chọn user → Xóa → confirm</t>
-  </si>
-  <si>
-    <t>User soft-delete</t>
-  </si>
-  <si>
-    <t>TC-079</t>
-  </si>
-  <si>
-    <t>IV.1.8</t>
-  </si>
-  <si>
-    <t>Giới hạn quyền cho đơn vị</t>
-  </si>
-  <si>
-    <t>Chọn đơn vị → Giới hạn quyền → chọn rights → Lưu</t>
-  </si>
-  <si>
-    <t>Quyền tối đa cho đơn vị set, user trong đơn vị không vượt quyền</t>
-  </si>
-  <si>
-    <t>HDSD có, code chưa implement — Phase 2</t>
+    <t>Defer Phase 2 — cần schema permission model mới</t>
   </si>
   <si>
     <t>TC-080</t>
@@ -1686,7 +1683,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1705,17 +1702,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
+        <fgColor rgb="FFE5E7EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFEE2E2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE5E7EB"/>
       </patternFill>
     </fill>
   </fills>
@@ -1753,7 +1745,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1768,9 +1760,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2499,69 +2488,69 @@
       <c r="G12" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>89</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>17</v>
@@ -2575,25 +2564,25 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>17</v>
@@ -2607,25 +2596,25 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="F16" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>17</v>
@@ -2639,217 +2628,217 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="H18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="F20" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="G20" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="H20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J20" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="F21" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="H21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J21" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D22" s="2" t="s">
+      <c r="E22" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="F22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="H22" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J22" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D23" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>145</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>17</v>
@@ -2863,185 +2852,185 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D24" s="2" t="s">
+      <c r="E24" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="G24" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="H24" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J24" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C25" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D25" s="2" t="s">
+      <c r="E25" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="E25" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="F25" s="2" t="s">
+      <c r="G25" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="H25" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J25" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D26" s="2" t="s">
+      <c r="E26" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="F26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="H26" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J26" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C27" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>28</v>
       </c>
       <c r="F27" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="H27" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J27" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="E28" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="G28" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="H28" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J28" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="C29" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D29" s="2" t="s">
+      <c r="E29" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="G29" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>183</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>17</v>
@@ -3055,25 +3044,25 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="C30" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D30" s="2" t="s">
+      <c r="E30" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="F30" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="G30" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>189</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>17</v>
@@ -3087,57 +3076,57 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="C31" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D31" s="2" t="s">
+      <c r="E31" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="F31" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="G31" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="H31" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J31" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I31" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="E32" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="F32" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="G32" s="2" t="s">
         <v>202</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>203</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>17</v>
@@ -3151,25 +3140,25 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C33" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="D33" s="2" t="s">
+      <c r="E33" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="F33" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>208</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>209</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>17</v>
@@ -3183,25 +3172,25 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="C34" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="D34" s="2" t="s">
+      <c r="E34" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F34" s="2" t="s">
+      <c r="G34" s="2" t="s">
         <v>213</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>214</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>17</v>
@@ -3215,57 +3204,57 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="D35" s="2" t="s">
+      <c r="E35" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="F35" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="G35" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="H35" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J35" s="2" t="s">
         <v>220</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="D36" s="2" t="s">
+      <c r="E36" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="F36" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G36" s="2" t="s">
         <v>225</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>226</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>17</v>
@@ -3279,25 +3268,25 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="C37" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C37" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="D37" s="2" t="s">
+      <c r="E37" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F37" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="F37" s="2" t="s">
+      <c r="G37" s="2" t="s">
         <v>230</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>231</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>17</v>
@@ -3311,25 +3300,25 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="C38" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="D38" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="F38" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="G38" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>237</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>17</v>
@@ -3343,25 +3332,25 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="C39" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="D39" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="E39" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="F39" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="F39" s="2" t="s">
+      <c r="G39" s="2" t="s">
         <v>243</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>244</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>17</v>
@@ -3375,25 +3364,25 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="C40" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D40" s="2" t="s">
+      <c r="E40" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="E40" s="2" t="s">
-        <v>248</v>
-      </c>
       <c r="F40" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>208</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>209</v>
       </c>
       <c r="H40" s="3" t="s">
         <v>17</v>
@@ -3407,25 +3396,25 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="C41" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D41" s="2" t="s">
+      <c r="E41" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="E41" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="F41" s="2" t="s">
+      <c r="G41" s="2" t="s">
         <v>252</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>253</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>17</v>
@@ -3439,25 +3428,25 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="C42" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="C42" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D42" s="2" t="s">
+      <c r="E42" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="E42" s="2" t="s">
-        <v>257</v>
-      </c>
       <c r="F42" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>17</v>
@@ -3471,25 +3460,25 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="C43" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D43" s="2" t="s">
+      <c r="E43" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="E43" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>261</v>
-      </c>
       <c r="G43" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>17</v>
@@ -3503,25 +3492,25 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="C44" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D44" s="2" t="s">
+      <c r="E44" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>264</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>265</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>17</v>
@@ -3535,25 +3524,25 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="C45" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="C45" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D45" s="2" t="s">
+      <c r="E45" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="F45" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="G45" s="2" t="s">
         <v>269</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>270</v>
       </c>
       <c r="H45" s="3" t="s">
         <v>17</v>
@@ -3567,89 +3556,89 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="C46" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="C46" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D46" s="2" t="s">
+      <c r="E46" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="E46" s="2" t="s">
+      <c r="F46" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="G46" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="H46" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J46" s="2" t="s">
         <v>276</v>
-      </c>
-      <c r="H46" s="5" t="s">
-        <v>277</v>
-      </c>
-      <c r="I46" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J46" s="2" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="E47" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="C47" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D47" s="2" t="s">
+      <c r="F47" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="E47" s="2" t="s">
+      <c r="G47" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J47" s="2" t="s">
         <v>282</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="H47" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="I47" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J47" s="2" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="E48" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="C48" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D48" s="2" t="s">
+      <c r="F48" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="E48" s="2" t="s">
+      <c r="G48" s="2" t="s">
         <v>288</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>290</v>
       </c>
       <c r="H48" s="3" t="s">
         <v>17</v>
@@ -3663,25 +3652,25 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="E49" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="C49" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D49" s="2" t="s">
+      <c r="F49" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G49" s="2" t="s">
         <v>293</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>295</v>
       </c>
       <c r="H49" s="3" t="s">
         <v>17</v>
@@ -3695,25 +3684,25 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>296</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>298</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>28</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="H50" s="3" t="s">
         <v>17</v>
@@ -3727,25 +3716,25 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="E51" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F51" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="C51" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D51" s="2" t="s">
+      <c r="G51" s="2" t="s">
         <v>303</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>305</v>
       </c>
       <c r="H51" s="3" t="s">
         <v>17</v>
@@ -3759,25 +3748,25 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="D52" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="E52" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="D52" s="2" t="s">
+      <c r="F52" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="E52" s="2" t="s">
+      <c r="G52" s="2" t="s">
         <v>310</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>312</v>
       </c>
       <c r="H52" s="3" t="s">
         <v>17</v>
@@ -3791,25 +3780,25 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="E53" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="C53" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D53" s="2" t="s">
+      <c r="F53" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="E53" s="2" t="s">
+      <c r="G53" s="2" t="s">
         <v>316</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>318</v>
       </c>
       <c r="H53" s="3" t="s">
         <v>17</v>
@@ -3823,25 +3812,25 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="E54" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F54" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="C54" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D54" s="2" t="s">
+      <c r="G54" s="2" t="s">
         <v>321</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>323</v>
       </c>
       <c r="H54" s="3" t="s">
         <v>17</v>
@@ -3855,25 +3844,25 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="D55" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="E55" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F55" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="C55" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D55" s="2" t="s">
+      <c r="G55" s="2" t="s">
         <v>326</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>328</v>
       </c>
       <c r="H55" s="3" t="s">
         <v>17</v>
@@ -3887,25 +3876,25 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="E56" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="C56" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D56" s="2" t="s">
+      <c r="F56" s="2" t="s">
         <v>331</v>
       </c>
-      <c r="E56" s="2" t="s">
+      <c r="G56" s="2" t="s">
         <v>332</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>334</v>
       </c>
       <c r="H56" s="3" t="s">
         <v>17</v>
@@ -3919,25 +3908,25 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="F57" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="B57" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D57" s="2" t="s">
+      <c r="G57" s="2" t="s">
         <v>336</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="G57" s="2" t="s">
-        <v>338</v>
       </c>
       <c r="H57" s="3" t="s">
         <v>17</v>
@@ -3951,25 +3940,25 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="D58" s="2" t="s">
         <v>340</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>342</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>28</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="H58" s="3" t="s">
         <v>17</v>
@@ -3983,25 +3972,25 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="E59" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="F59" s="2" t="s">
         <v>346</v>
       </c>
-      <c r="C59" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D59" s="2" t="s">
+      <c r="G59" s="2" t="s">
         <v>347</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="G59" s="2" t="s">
-        <v>349</v>
       </c>
       <c r="H59" s="3" t="s">
         <v>17</v>
@@ -4015,25 +4004,25 @@
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D60" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="E60" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="C60" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D60" s="2" t="s">
+      <c r="F60" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="E60" s="2" t="s">
+      <c r="G60" s="2" t="s">
         <v>353</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>355</v>
       </c>
       <c r="H60" s="3" t="s">
         <v>17</v>
@@ -4047,57 +4036,57 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D61" s="2" t="s">
         <v>356</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="E61" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D61" s="2" t="s">
+      <c r="F61" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="E61" s="2" t="s">
+      <c r="G61" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J61" s="2" t="s">
         <v>359</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="G61" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="H61" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I61" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J61" s="2" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D62" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="E62" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="C62" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D62" s="2" t="s">
+      <c r="F62" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="E62" s="2" t="s">
+      <c r="G62" s="2" t="s">
         <v>365</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="G62" s="2" t="s">
-        <v>367</v>
       </c>
       <c r="H62" s="3" t="s">
         <v>17</v>
@@ -4111,25 +4100,25 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="E63" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="C63" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D63" s="2" t="s">
+      <c r="F63" s="2" t="s">
         <v>370</v>
       </c>
-      <c r="E63" s="2" t="s">
+      <c r="G63" s="2" t="s">
         <v>371</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="G63" s="2" t="s">
-        <v>373</v>
       </c>
       <c r="H63" s="3" t="s">
         <v>17</v>
@@ -4143,25 +4132,25 @@
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>374</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="E64" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F64" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="C64" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D64" s="2" t="s">
+      <c r="G64" s="2" t="s">
         <v>376</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="G64" s="2" t="s">
-        <v>378</v>
       </c>
       <c r="H64" s="3" t="s">
         <v>17</v>
@@ -4175,25 +4164,25 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="E65" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="C65" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D65" s="2" t="s">
+      <c r="F65" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="E65" s="2" t="s">
+      <c r="G65" s="2" t="s">
         <v>382</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="G65" s="2" t="s">
-        <v>384</v>
       </c>
       <c r="H65" s="3" t="s">
         <v>17</v>
@@ -4207,217 +4196,217 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="E66" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="C66" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D66" s="2" t="s">
+      <c r="F66" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="E66" s="2" t="s">
+      <c r="G66" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="F66" s="2" t="s">
+      <c r="H66" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J66" s="2" t="s">
         <v>389</v>
-      </c>
-      <c r="G66" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="H66" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I66" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J66" s="2" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D67" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="E67" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="C67" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D67" s="2" t="s">
+      <c r="F67" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="E67" s="2" t="s">
+      <c r="G67" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="F67" s="2" t="s">
+      <c r="H67" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J67" s="2" t="s">
         <v>396</v>
-      </c>
-      <c r="G67" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="H67" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="I67" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J67" s="2" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D68" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="E68" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="F68" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="C68" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D68" s="2" t="s">
+      <c r="G68" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="E68" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="F68" s="2" t="s">
+      <c r="H68" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J68" s="2" t="s">
         <v>402</v>
-      </c>
-      <c r="G68" s="2" t="s">
-        <v>403</v>
-      </c>
-      <c r="H68" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="I68" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J68" s="2" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D69" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="E69" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="C69" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D69" s="2" t="s">
+      <c r="F69" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="E69" s="2" t="s">
+      <c r="G69" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="F69" s="2" t="s">
+      <c r="H69" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J69" s="2" t="s">
         <v>409</v>
-      </c>
-      <c r="G69" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="H69" s="5" t="s">
-        <v>277</v>
-      </c>
-      <c r="I69" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J69" s="2" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D70" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="E70" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="C70" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D70" s="2" t="s">
+      <c r="F70" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E70" s="2" t="s">
+      <c r="G70" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="F70" s="2" t="s">
+      <c r="H70" s="4" t="s">
         <v>416</v>
       </c>
-      <c r="G70" s="2" t="s">
+      <c r="I70" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J70" s="2" t="s">
         <v>417</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>418</v>
-      </c>
-      <c r="I70" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J70" s="2" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D71" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="E71" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="C71" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D71" s="2" t="s">
+      <c r="F71" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="E71" s="2" t="s">
+      <c r="G71" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="F71" s="2" t="s">
+      <c r="H71" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I71" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J71" s="2" t="s">
         <v>424</v>
-      </c>
-      <c r="G71" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="H71" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="I71" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J71" s="2" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D72" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="E72" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="F72" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="C72" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D72" s="2" t="s">
+      <c r="G72" s="2" t="s">
         <v>429</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="G72" s="2" t="s">
-        <v>431</v>
       </c>
       <c r="H72" s="3" t="s">
         <v>17</v>
@@ -4431,25 +4420,25 @@
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C73" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="D73" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="C73" s="2" t="s">
+      <c r="E73" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F73" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="D73" s="2" t="s">
+      <c r="G73" s="2" t="s">
         <v>435</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>436</v>
-      </c>
-      <c r="G73" s="2" t="s">
-        <v>437</v>
       </c>
       <c r="H73" s="3" t="s">
         <v>17</v>
@@ -4463,25 +4452,25 @@
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D74" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="E74" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F74" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="C74" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D74" s="2" t="s">
+      <c r="G74" s="2" t="s">
         <v>440</v>
-      </c>
-      <c r="E74" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="F74" s="2" t="s">
-        <v>441</v>
-      </c>
-      <c r="G74" s="2" t="s">
-        <v>442</v>
       </c>
       <c r="H74" s="3" t="s">
         <v>17</v>
@@ -4495,25 +4484,25 @@
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D75" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="E75" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="C75" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D75" s="2" t="s">
+      <c r="F75" s="2" t="s">
         <v>445</v>
       </c>
-      <c r="E75" s="2" t="s">
+      <c r="G75" s="2" t="s">
         <v>446</v>
-      </c>
-      <c r="F75" s="2" t="s">
-        <v>447</v>
-      </c>
-      <c r="G75" s="2" t="s">
-        <v>448</v>
       </c>
       <c r="H75" s="3" t="s">
         <v>17</v>
@@ -4527,25 +4516,25 @@
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D76" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="E76" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="C76" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D76" s="2" t="s">
+      <c r="F76" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="E76" s="2" t="s">
+      <c r="G76" s="2" t="s">
         <v>452</v>
-      </c>
-      <c r="F76" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="G76" s="2" t="s">
-        <v>454</v>
       </c>
       <c r="H76" s="3" t="s">
         <v>17</v>
@@ -4559,89 +4548,89 @@
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D77" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="E77" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="C77" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D77" s="2" t="s">
+      <c r="F77" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="E77" s="2" t="s">
+      <c r="G77" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="F77" s="2" t="s">
+      <c r="H77" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I77" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J77" s="2" t="s">
         <v>459</v>
-      </c>
-      <c r="G77" s="2" t="s">
-        <v>460</v>
-      </c>
-      <c r="H77" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I77" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J77" s="2" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D78" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="E78" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="C78" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D78" s="2" t="s">
+      <c r="F78" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="E78" s="2" t="s">
+      <c r="G78" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="F78" s="2" t="s">
+      <c r="H78" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I78" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J78" s="2" t="s">
         <v>466</v>
-      </c>
-      <c r="G78" s="2" t="s">
-        <v>467</v>
-      </c>
-      <c r="H78" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I78" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J78" s="2" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D79" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="E79" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="C79" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D79" s="2" t="s">
+      <c r="F79" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="E79" s="2" t="s">
+      <c r="G79" s="2" t="s">
         <v>472</v>
-      </c>
-      <c r="F79" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="G79" s="2" t="s">
-        <v>474</v>
       </c>
       <c r="H79" s="3" t="s">
         <v>17</v>
@@ -4655,57 +4644,57 @@
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D80" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="E80" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F80" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="C80" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D80" s="2" t="s">
+      <c r="G80" s="2" t="s">
         <v>477</v>
       </c>
-      <c r="E80" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="F80" s="2" t="s">
+      <c r="H80" s="5" t="s">
         <v>478</v>
       </c>
-      <c r="G80" s="2" t="s">
+      <c r="I80" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J80" s="2" t="s">
         <v>479</v>
-      </c>
-      <c r="H80" s="5" t="s">
-        <v>277</v>
-      </c>
-      <c r="I80" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J80" s="2" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="B81" s="2" t="s">
         <v>481</v>
       </c>
-      <c r="B81" s="2" t="s">
+      <c r="C81" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D81" s="2" t="s">
         <v>482</v>
       </c>
-      <c r="C81" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D81" s="2" t="s">
+      <c r="E81" s="2" t="s">
         <v>483</v>
       </c>
-      <c r="E81" s="2" t="s">
+      <c r="F81" s="2" t="s">
         <v>484</v>
       </c>
-      <c r="F81" s="2" t="s">
+      <c r="G81" s="2" t="s">
         <v>485</v>
-      </c>
-      <c r="G81" s="2" t="s">
-        <v>486</v>
       </c>
       <c r="H81" s="3" t="s">
         <v>17</v>
@@ -4719,25 +4708,25 @@
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="B82" s="2" t="s">
         <v>487</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="C82" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D82" s="2" t="s">
         <v>488</v>
       </c>
-      <c r="C82" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D82" s="2" t="s">
+      <c r="E82" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F82" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="E82" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="F82" s="2" t="s">
+      <c r="G82" s="2" t="s">
         <v>490</v>
-      </c>
-      <c r="G82" s="2" t="s">
-        <v>491</v>
       </c>
       <c r="H82" s="3" t="s">
         <v>17</v>
@@ -4751,25 +4740,25 @@
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="B83" s="2" t="s">
         <v>492</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="C83" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D83" s="2" t="s">
         <v>493</v>
       </c>
-      <c r="C83" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D83" s="2" t="s">
+      <c r="E83" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F83" s="2" t="s">
         <v>494</v>
       </c>
-      <c r="E83" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="F83" s="2" t="s">
+      <c r="G83" s="2" t="s">
         <v>495</v>
-      </c>
-      <c r="G83" s="2" t="s">
-        <v>496</v>
       </c>
       <c r="H83" s="3" t="s">
         <v>17</v>
@@ -4783,25 +4772,25 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="B84" s="2" t="s">
         <v>497</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="C84" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D84" s="2" t="s">
         <v>498</v>
       </c>
-      <c r="C84" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D84" s="2" t="s">
+      <c r="E84" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F84" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="E84" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="F84" s="2" t="s">
+      <c r="G84" s="2" t="s">
         <v>500</v>
-      </c>
-      <c r="G84" s="2" t="s">
-        <v>501</v>
       </c>
       <c r="H84" s="3" t="s">
         <v>17</v>
@@ -4815,25 +4804,25 @@
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="B85" s="2" t="s">
         <v>502</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="C85" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D85" s="2" t="s">
         <v>503</v>
       </c>
-      <c r="C85" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D85" s="2" t="s">
+      <c r="E85" s="2" t="s">
         <v>504</v>
       </c>
-      <c r="E85" s="2" t="s">
+      <c r="F85" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="F85" s="2" t="s">
+      <c r="G85" s="2" t="s">
         <v>506</v>
-      </c>
-      <c r="G85" s="2" t="s">
-        <v>507</v>
       </c>
       <c r="H85" s="3" t="s">
         <v>17</v>
@@ -4847,25 +4836,25 @@
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="B86" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="C86" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D86" s="2" t="s">
         <v>509</v>
       </c>
-      <c r="C86" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D86" s="2" t="s">
+      <c r="E86" s="2" t="s">
         <v>510</v>
       </c>
-      <c r="E86" s="2" t="s">
+      <c r="F86" s="2" t="s">
         <v>511</v>
       </c>
-      <c r="F86" s="2" t="s">
+      <c r="G86" s="2" t="s">
         <v>512</v>
-      </c>
-      <c r="G86" s="2" t="s">
-        <v>513</v>
       </c>
       <c r="H86" s="3" t="s">
         <v>17</v>
@@ -4879,57 +4868,57 @@
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="B87" s="2" t="s">
         <v>514</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="C87" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D87" s="2" t="s">
         <v>515</v>
       </c>
-      <c r="C87" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D87" s="2" t="s">
+      <c r="E87" s="2" t="s">
         <v>516</v>
       </c>
-      <c r="E87" s="2" t="s">
+      <c r="F87" s="2" t="s">
         <v>517</v>
       </c>
-      <c r="F87" s="2" t="s">
+      <c r="G87" s="2" t="s">
         <v>518</v>
       </c>
-      <c r="G87" s="2" t="s">
+      <c r="H87" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I87" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J87" s="2" t="s">
         <v>519</v>
-      </c>
-      <c r="H87" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I87" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J87" s="2" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="B88" s="2" t="s">
         <v>521</v>
       </c>
-      <c r="B88" s="2" t="s">
+      <c r="C88" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D88" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="C88" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D88" s="2" t="s">
+      <c r="E88" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F88" s="2" t="s">
         <v>523</v>
       </c>
-      <c r="E88" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="F88" s="2" t="s">
+      <c r="G88" s="2" t="s">
         <v>524</v>
-      </c>
-      <c r="G88" s="2" t="s">
-        <v>525</v>
       </c>
       <c r="H88" s="3" t="s">
         <v>17</v>
@@ -4943,25 +4932,25 @@
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B89" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="C89" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D89" s="2" t="s">
         <v>527</v>
       </c>
-      <c r="C89" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D89" s="2" t="s">
+      <c r="E89" s="2" t="s">
         <v>528</v>
       </c>
-      <c r="E89" s="2" t="s">
+      <c r="F89" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="F89" s="2" t="s">
+      <c r="G89" s="2" t="s">
         <v>530</v>
-      </c>
-      <c r="G89" s="2" t="s">
-        <v>531</v>
       </c>
       <c r="H89" s="3" t="s">
         <v>17</v>
@@ -4975,25 +4964,25 @@
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B90" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="B90" s="2" t="s">
+      <c r="C90" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D90" s="2" t="s">
         <v>533</v>
       </c>
-      <c r="C90" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D90" s="2" t="s">
+      <c r="E90" s="2" t="s">
         <v>534</v>
       </c>
-      <c r="E90" s="2" t="s">
+      <c r="F90" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="F90" s="2" t="s">
+      <c r="G90" s="2" t="s">
         <v>536</v>
-      </c>
-      <c r="G90" s="2" t="s">
-        <v>537</v>
       </c>
       <c r="H90" s="3" t="s">
         <v>17</v>
@@ -5007,25 +4996,25 @@
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="B91" s="2" t="s">
         <v>538</v>
       </c>
-      <c r="B91" s="2" t="s">
+      <c r="C91" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D91" s="2" t="s">
         <v>539</v>
       </c>
-      <c r="C91" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D91" s="2" t="s">
+      <c r="E91" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F91" s="2" t="s">
         <v>540</v>
       </c>
-      <c r="E91" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="F91" s="2" t="s">
+      <c r="G91" s="2" t="s">
         <v>541</v>
-      </c>
-      <c r="G91" s="2" t="s">
-        <v>542</v>
       </c>
       <c r="H91" s="3" t="s">
         <v>17</v>
@@ -5039,25 +5028,25 @@
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="B92" s="2" t="s">
         <v>543</v>
       </c>
-      <c r="B92" s="2" t="s">
+      <c r="C92" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D92" s="2" t="s">
         <v>544</v>
       </c>
-      <c r="C92" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D92" s="2" t="s">
+      <c r="E92" s="2" t="s">
         <v>545</v>
       </c>
-      <c r="E92" s="2" t="s">
-        <v>546</v>
-      </c>
       <c r="F92" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="G92" s="2" t="s">
         <v>530</v>
-      </c>
-      <c r="G92" s="2" t="s">
-        <v>531</v>
       </c>
       <c r="H92" s="3" t="s">
         <v>17</v>
@@ -5071,26 +5060,26 @@
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="B93" s="2" t="s">
         <v>547</v>
       </c>
-      <c r="B93" s="2" t="s">
+      <c r="C93" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D93" s="2" t="s">
         <v>548</v>
       </c>
-      <c r="C93" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D93" s="2" t="s">
+      <c r="E93" s="2" t="s">
         <v>549</v>
       </c>
-      <c r="E93" s="2" t="s">
-        <v>550</v>
-      </c>
       <c r="F93" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="G93" s="2" t="s">
         <v>536</v>
       </c>
-      <c r="G93" s="2" t="s">
-        <v>537</v>
-      </c>
       <c r="H93" s="3" t="s">
         <v>17</v>
       </c>
@@ -5098,7 +5087,7 @@
         <v>18</v>
       </c>
       <c r="J93" s="2" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: cập nhật kết quả test_theo_hdsd_cu (UAT thực tế)
</commit_message>
<xml_diff>
--- a/docs/test_theo_hdsd_cu.xlsx
+++ b/docs/test_theo_hdsd_cu.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1457C201-E7AF-4C94-B692-F253E6B7DE34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Test cases" state="visible" r:id="rId4"/>
+    <sheet name="Test cases" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -1666,24 +1670,28 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1710,6 +1718,12 @@
         <fgColor rgb="FFFEE2E2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -1720,10 +1734,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1745,7 +1767,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1760,6 +1782,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2100,9 +2125,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J93"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
@@ -2114,7 +2139,7 @@
     <col min="10" max="10" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2146,7 +2171,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2178,7 +2203,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>20</v>
       </c>
@@ -2210,7 +2235,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>25</v>
       </c>
@@ -2242,7 +2267,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>31</v>
       </c>
@@ -2274,7 +2299,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>36</v>
       </c>
@@ -2306,7 +2331,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>40</v>
       </c>
@@ -2338,7 +2363,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>47</v>
       </c>
@@ -2370,7 +2395,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>53</v>
       </c>
@@ -2402,7 +2427,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>58</v>
       </c>
@@ -2434,7 +2459,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>63</v>
       </c>
@@ -2466,7 +2491,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>69</v>
       </c>
@@ -2498,7 +2523,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>76</v>
       </c>
@@ -2530,7 +2555,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>84</v>
       </c>
@@ -2562,7 +2587,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>89</v>
       </c>
@@ -2594,7 +2619,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>93</v>
       </c>
@@ -2626,7 +2651,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>99</v>
       </c>
@@ -2658,7 +2683,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>106</v>
       </c>
@@ -2690,7 +2715,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>113</v>
       </c>
@@ -2722,7 +2747,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>120</v>
       </c>
@@ -2754,7 +2779,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>127</v>
       </c>
@@ -2786,7 +2811,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>134</v>
       </c>
@@ -2818,7 +2843,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>140</v>
       </c>
@@ -2850,7 +2875,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>145</v>
       </c>
@@ -2882,7 +2907,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>152</v>
       </c>
@@ -2914,7 +2939,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>158</v>
       </c>
@@ -2946,7 +2971,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>164</v>
       </c>
@@ -2978,7 +3003,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>170</v>
       </c>
@@ -3010,7 +3035,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>177</v>
       </c>
@@ -3042,7 +3067,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>183</v>
       </c>
@@ -3074,7 +3099,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>189</v>
       </c>
@@ -3106,7 +3131,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>196</v>
       </c>
@@ -3138,7 +3163,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>203</v>
       </c>
@@ -3170,7 +3195,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>209</v>
       </c>
@@ -3202,7 +3227,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>214</v>
       </c>
@@ -3234,7 +3259,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>221</v>
       </c>
@@ -3266,7 +3291,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>226</v>
       </c>
@@ -3298,7 +3323,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>231</v>
       </c>
@@ -3330,7 +3355,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>237</v>
       </c>
@@ -3362,7 +3387,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>244</v>
       </c>
@@ -3394,7 +3419,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>248</v>
       </c>
@@ -3426,7 +3451,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>253</v>
       </c>
@@ -3458,7 +3483,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>257</v>
       </c>
@@ -3490,7 +3515,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>261</v>
       </c>
@@ -3522,7 +3547,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>265</v>
       </c>
@@ -3554,7 +3579,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>270</v>
       </c>
@@ -3586,7 +3611,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>277</v>
       </c>
@@ -3618,7 +3643,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>283</v>
       </c>
@@ -3650,7 +3675,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>289</v>
       </c>
@@ -3682,7 +3707,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>294</v>
       </c>
@@ -3714,7 +3739,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>299</v>
       </c>
@@ -3746,7 +3771,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>304</v>
       </c>
@@ -3778,7 +3803,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>311</v>
       </c>
@@ -3810,7 +3835,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>317</v>
       </c>
@@ -3842,7 +3867,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>322</v>
       </c>
@@ -3874,7 +3899,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>327</v>
       </c>
@@ -3906,7 +3931,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>333</v>
       </c>
@@ -3938,7 +3963,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>337</v>
       </c>
@@ -3970,7 +3995,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>343</v>
       </c>
@@ -4002,7 +4027,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>348</v>
       </c>
@@ -4034,7 +4059,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>354</v>
       </c>
@@ -4066,7 +4091,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>360</v>
       </c>
@@ -4098,7 +4123,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>366</v>
       </c>
@@ -4130,7 +4155,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>372</v>
       </c>
@@ -4162,7 +4187,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>377</v>
       </c>
@@ -4194,7 +4219,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>383</v>
       </c>
@@ -4226,7 +4251,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>390</v>
       </c>
@@ -4258,7 +4283,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>397</v>
       </c>
@@ -4290,7 +4315,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>403</v>
       </c>
@@ -4322,7 +4347,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>410</v>
       </c>
@@ -4350,11 +4375,11 @@
       <c r="I70" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J70" s="2" t="s">
+      <c r="J70" s="6" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>418</v>
       </c>
@@ -4386,7 +4411,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>425</v>
       </c>
@@ -4418,7 +4443,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>430</v>
       </c>
@@ -4450,7 +4475,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>436</v>
       </c>
@@ -4482,7 +4507,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>441</v>
       </c>
@@ -4514,7 +4539,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>447</v>
       </c>
@@ -4546,7 +4571,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>453</v>
       </c>
@@ -4578,7 +4603,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>460</v>
       </c>
@@ -4610,7 +4635,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>467</v>
       </c>
@@ -4642,7 +4667,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>473</v>
       </c>
@@ -4670,11 +4695,11 @@
       <c r="I80" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J80" s="2" t="s">
+      <c r="J80" s="6" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>480</v>
       </c>
@@ -4706,7 +4731,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>486</v>
       </c>
@@ -4738,7 +4763,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>491</v>
       </c>
@@ -4770,7 +4795,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>496</v>
       </c>
@@ -4802,7 +4827,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>501</v>
       </c>
@@ -4834,7 +4859,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>507</v>
       </c>
@@ -4866,7 +4891,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>513</v>
       </c>
@@ -4898,7 +4923,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>520</v>
       </c>
@@ -4930,7 +4955,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>525</v>
       </c>
@@ -4962,7 +4987,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>531</v>
       </c>
@@ -4994,7 +5019,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>537</v>
       </c>
@@ -5026,7 +5051,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>542</v>
       </c>
@@ -5058,7 +5083,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>546</v>
       </c>
@@ -5091,8 +5116,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J93"/>
+  <autoFilter ref="A1:J93" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>